<commit_message>
feat(schema): normalize CBSA geography data
  Store metro metadata once and reference it from business
  geography and tract context. Preserve raw outlying text.
</commit_message>
<xml_diff>
--- a/data/Variable_Codebook.xlsx
+++ b/data/Variable_Codebook.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahesh\Documents\Research\Gay Bars\Ownership\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9f3ba96d5af42d13/Desktop/Research_summer_2026/research_business_project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA52D1A-D0D2-4899-983D-63991D59F62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{9FA52D1A-D0D2-4899-983D-63991D59F62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{513C4CB1-14C3-48E9-B397-DCFC43CFBE13}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7FE0A9C2-515F-4A73-9198-FF38E2ED6523}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{7FE0A9C2-515F-4A73-9198-FF38E2ED6523}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1088,9 +1088,6 @@
     <t>Whether Geocode Was Done Using Google (Google) or TigerLine (SAS)</t>
   </si>
   <si>
-    <t>Coordinate in USA_Contiguous_Albers_Equal_Area_Conic Projection</t>
-  </si>
-  <si>
     <t>When using Google, whether exact  (ROOFTOP) or approximate (RANGE_INTERPOLATED) geocode</t>
   </si>
   <si>
@@ -1212,6 +1209,9 @@
   </si>
   <si>
     <t>Non-censal year values are interpolated between Census or ACS Years</t>
+  </si>
+  <si>
+    <t>Coordinate in USA_Contiguous_Albers_Equal_Area_Conic Projection (102003)</t>
   </si>
 </sst>
 </file>
@@ -1604,16 +1604,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC58AD8-B993-4CAA-A450-B473FEBBEBD3}">
   <dimension ref="A1:F230"/>
-  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="16.85546875" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="107.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="116.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="16.81640625" customWidth="1"/>
+    <col min="4" max="4" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="107.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="116.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1624,7 +1624,7 @@
         <v>317</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -1633,7 +1633,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>136</v>
       </c>
@@ -1645,10 +1645,10 @@
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>137</v>
       </c>
@@ -1660,13 +1660,13 @@
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -1684,7 +1684,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -1714,7 +1714,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>185</v>
       </c>
@@ -1725,13 +1725,13 @@
         <v>314</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -1764,7 +1764,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
@@ -1779,10 +1779,10 @@
         <v>307</v>
       </c>
       <c r="F10" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>36</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>42</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>44</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>46</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>48</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>50</v>
       </c>
@@ -1872,7 +1872,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>52</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -1905,7 +1905,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>57</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>59</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>61</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>63</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>65</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>67</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>69</v>
       </c>
@@ -2010,7 +2010,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>71</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>73</v>
       </c>
@@ -2040,7 +2040,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>81</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>83</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>84</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>86</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>88</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>89</v>
       </c>
@@ -2140,7 +2140,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>138</v>
       </c>
@@ -2152,10 +2152,10 @@
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>139</v>
       </c>
@@ -2169,10 +2169,10 @@
         <v>321</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>176</v>
       </c>
@@ -2184,10 +2184,10 @@
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>177</v>
       </c>
@@ -2199,10 +2199,10 @@
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>182</v>
       </c>
@@ -2214,10 +2214,10 @@
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>186</v>
       </c>
@@ -2229,10 +2229,10 @@
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>187</v>
       </c>
@@ -2244,10 +2244,10 @@
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>188</v>
       </c>
@@ -2259,10 +2259,10 @@
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>191</v>
       </c>
@@ -2274,10 +2274,10 @@
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>192</v>
       </c>
@@ -2289,10 +2289,10 @@
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>193</v>
       </c>
@@ -2304,10 +2304,10 @@
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>153</v>
       </c>
@@ -2318,16 +2318,16 @@
         <v>314</v>
       </c>
       <c r="D45" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F45" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>210</v>
       </c>
@@ -2338,16 +2338,16 @@
         <v>314</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F46" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>154</v>
       </c>
@@ -2361,13 +2361,13 @@
         <v>324</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F47" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>224</v>
       </c>
@@ -2381,13 +2381,13 @@
         <v>324</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F48" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>155</v>
       </c>
@@ -2401,13 +2401,13 @@
         <v>325</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F49" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>227</v>
       </c>
@@ -2421,13 +2421,13 @@
         <v>325</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F50" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>156</v>
       </c>
@@ -2441,13 +2441,13 @@
         <v>327</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F51" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>214</v>
       </c>
@@ -2461,13 +2461,13 @@
         <v>327</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F52" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>157</v>
       </c>
@@ -2481,13 +2481,13 @@
         <v>326</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F53" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>209</v>
       </c>
@@ -2501,13 +2501,13 @@
         <v>326</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F54" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>158</v>
       </c>
@@ -2527,7 +2527,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>216</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>159</v>
       </c>
@@ -2561,13 +2561,13 @@
         <v>330</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F57" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>228</v>
       </c>
@@ -2581,13 +2581,13 @@
         <v>330</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F58" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>160</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>222</v>
       </c>
@@ -2627,7 +2627,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>161</v>
       </c>
@@ -2647,7 +2647,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>208</v>
       </c>
@@ -2667,7 +2667,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>169</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>201</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>170</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>215</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>171</v>
       </c>
@@ -2761,13 +2761,13 @@
         <v>342</v>
       </c>
       <c r="E67" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F67" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>200</v>
       </c>
@@ -2781,13 +2781,13 @@
         <v>342</v>
       </c>
       <c r="E68" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F68" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>172</v>
       </c>
@@ -2801,13 +2801,13 @@
         <v>343</v>
       </c>
       <c r="E69" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F69" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>218</v>
       </c>
@@ -2821,13 +2821,13 @@
         <v>343</v>
       </c>
       <c r="E70" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F70" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>173</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>226</v>
       </c>
@@ -2867,7 +2867,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>174</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>175</v>
       </c>
@@ -2907,7 +2907,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>211</v>
       </c>
@@ -2927,7 +2927,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>302</v>
       </c>
@@ -2939,13 +2939,13 @@
       </c>
       <c r="D76" s="2"/>
       <c r="E76" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F76" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>204</v>
       </c>
@@ -2959,13 +2959,13 @@
         <v>302</v>
       </c>
       <c r="E77" t="s">
+        <v>380</v>
+      </c>
+      <c r="F77" t="s">
         <v>381</v>
       </c>
-      <c r="F77" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>205</v>
       </c>
@@ -2979,13 +2979,13 @@
         <v>302</v>
       </c>
       <c r="E78" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F78" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>296</v>
       </c>
@@ -2997,13 +2997,13 @@
       </c>
       <c r="D79" s="2"/>
       <c r="E79" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F79" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>225</v>
       </c>
@@ -3017,13 +3017,13 @@
         <v>296</v>
       </c>
       <c r="E80" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F80" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>299</v>
       </c>
@@ -3035,13 +3035,13 @@
       </c>
       <c r="D81" s="2"/>
       <c r="E81" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F81" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>229</v>
       </c>
@@ -3055,13 +3055,13 @@
         <v>299</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F82" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>300</v>
       </c>
@@ -3073,13 +3073,13 @@
       </c>
       <c r="D83" s="2"/>
       <c r="E83" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F83" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>230</v>
       </c>
@@ -3093,13 +3093,13 @@
         <v>300</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F84" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
         <v>303</v>
       </c>
@@ -3111,13 +3111,13 @@
       </c>
       <c r="D85" s="3"/>
       <c r="E85" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F85" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>196</v>
       </c>
@@ -3131,13 +3131,13 @@
         <v>303</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F86" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>297</v>
       </c>
@@ -3149,13 +3149,13 @@
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F87" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>197</v>
       </c>
@@ -3169,13 +3169,13 @@
         <v>297</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F88" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>298</v>
       </c>
@@ -3187,13 +3187,13 @@
       </c>
       <c r="D89" s="2"/>
       <c r="E89" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F89" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>232</v>
       </c>
@@ -3205,13 +3205,13 @@
       </c>
       <c r="D90" s="2"/>
       <c r="E90" t="s">
+        <v>350</v>
+      </c>
+      <c r="F90" t="s">
         <v>351</v>
       </c>
-      <c r="F90" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>234</v>
       </c>
@@ -3226,7 +3226,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>235</v>
       </c>
@@ -3238,10 +3238,10 @@
       </c>
       <c r="D92" s="2"/>
       <c r="E92" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>236</v>
       </c>
@@ -3253,10 +3253,10 @@
       </c>
       <c r="D93" s="2"/>
       <c r="E93" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>278</v>
       </c>
@@ -3268,10 +3268,10 @@
       </c>
       <c r="D94" s="2"/>
       <c r="E94" s="2" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>195</v>
       </c>
@@ -3282,25 +3282,25 @@
         <v>314</v>
       </c>
       <c r="D95" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="E95" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="E95" s="2" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
       <c r="E96" s="2"/>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" s="4" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>16</v>
       </c>
@@ -3313,7 +3313,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>9</v>
       </c>
@@ -3329,7 +3329,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>22</v>
       </c>
@@ -3345,7 +3345,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>25</v>
       </c>
@@ -3359,7 +3359,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>28</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>31</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>33</v>
       </c>
@@ -3395,7 +3395,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>38</v>
       </c>
@@ -3406,7 +3406,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>40</v>
       </c>
@@ -3420,7 +3420,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>12</v>
       </c>
@@ -3435,7 +3435,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>14</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>90</v>
       </c>
@@ -3461,7 +3461,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>92</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>93</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>94</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>96</v>
       </c>
@@ -3517,7 +3517,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>97</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>98</v>
       </c>
@@ -3545,7 +3545,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>99</v>
       </c>
@@ -3559,7 +3559,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>101</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>121</v>
       </c>
@@ -3587,7 +3587,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>122</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>123</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>124</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>125</v>
       </c>
@@ -3643,7 +3643,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>126</v>
       </c>
@@ -3657,7 +3657,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
         <v>127</v>
       </c>
@@ -3671,7 +3671,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>178</v>
       </c>
@@ -3679,7 +3679,7 @@
       <c r="C126" s="2"/>
       <c r="D126" s="2"/>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
         <v>179</v>
       </c>
@@ -3687,7 +3687,7 @@
       <c r="C127" s="2"/>
       <c r="D127" s="2"/>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>180</v>
       </c>
@@ -3695,7 +3695,7 @@
       <c r="C128" s="2"/>
       <c r="D128" s="2"/>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
         <v>181</v>
       </c>
@@ -3703,7 +3703,7 @@
       <c r="C129" s="2"/>
       <c r="D129" s="2"/>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>183</v>
       </c>
@@ -3711,7 +3711,7 @@
       <c r="C130" s="2"/>
       <c r="D130" s="2"/>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>184</v>
       </c>
@@ -3719,7 +3719,7 @@
       <c r="C131" s="2"/>
       <c r="D131" s="2"/>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>189</v>
       </c>
@@ -3727,7 +3727,7 @@
       <c r="C132" s="2"/>
       <c r="D132" s="2"/>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>190</v>
       </c>
@@ -3735,7 +3735,7 @@
       <c r="C133" s="2"/>
       <c r="D133" s="2"/>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
         <v>194</v>
       </c>
@@ -3743,7 +3743,7 @@
       <c r="C134" s="2"/>
       <c r="D134" s="2"/>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
         <v>231</v>
       </c>
@@ -3755,7 +3755,7 @@
       </c>
       <c r="D135" s="2"/>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
         <v>75</v>
       </c>
@@ -3773,7 +3773,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>78</v>
       </c>
@@ -3791,7 +3791,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>237</v>
       </c>
@@ -3799,7 +3799,7 @@
       <c r="C138" s="2"/>
       <c r="D138" s="2"/>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
         <v>238</v>
       </c>
@@ -3807,7 +3807,7 @@
       <c r="C139" s="2"/>
       <c r="D139" s="2"/>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>239</v>
       </c>
@@ -3815,7 +3815,7 @@
       <c r="C140" s="2"/>
       <c r="D140" s="2"/>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
         <v>240</v>
       </c>
@@ -3823,7 +3823,7 @@
       <c r="C141" s="2"/>
       <c r="D141" s="2"/>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142" s="2" t="s">
         <v>241</v>
       </c>
@@ -3831,7 +3831,7 @@
       <c r="C142" s="2"/>
       <c r="D142" s="2"/>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
         <v>242</v>
       </c>
@@ -3839,7 +3839,7 @@
       <c r="C143" s="2"/>
       <c r="D143" s="2"/>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
         <v>243</v>
       </c>
@@ -3847,7 +3847,7 @@
       <c r="C144" s="2"/>
       <c r="D144" s="2"/>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
         <v>244</v>
       </c>
@@ -3855,7 +3855,7 @@
       <c r="C145" s="2"/>
       <c r="D145" s="2"/>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
         <v>245</v>
       </c>
@@ -3863,7 +3863,7 @@
       <c r="C146" s="2"/>
       <c r="D146" s="2"/>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" s="2" t="s">
         <v>246</v>
       </c>
@@ -3871,7 +3871,7 @@
       <c r="C147" s="2"/>
       <c r="D147" s="2"/>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" s="2" t="s">
         <v>247</v>
       </c>
@@ -3879,7 +3879,7 @@
       <c r="C148" s="2"/>
       <c r="D148" s="2"/>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
         <v>248</v>
       </c>
@@ -3887,7 +3887,7 @@
       <c r="C149" s="2"/>
       <c r="D149" s="2"/>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>249</v>
       </c>
@@ -3895,7 +3895,7 @@
       <c r="C150" s="2"/>
       <c r="D150" s="2"/>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
         <v>250</v>
       </c>
@@ -3903,7 +3903,7 @@
       <c r="C151" s="2"/>
       <c r="D151" s="2"/>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
         <v>251</v>
       </c>
@@ -3911,7 +3911,7 @@
       <c r="C152" s="2"/>
       <c r="D152" s="2"/>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
         <v>252</v>
       </c>
@@ -3919,7 +3919,7 @@
       <c r="C153" s="2"/>
       <c r="D153" s="2"/>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
         <v>253</v>
       </c>
@@ -3927,7 +3927,7 @@
       <c r="C154" s="2"/>
       <c r="D154" s="2"/>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
         <v>254</v>
       </c>
@@ -3935,7 +3935,7 @@
       <c r="C155" s="2"/>
       <c r="D155" s="2"/>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
         <v>255</v>
       </c>
@@ -3943,7 +3943,7 @@
       <c r="C156" s="2"/>
       <c r="D156" s="2"/>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
         <v>256</v>
       </c>
@@ -3951,7 +3951,7 @@
       <c r="C157" s="2"/>
       <c r="D157" s="2"/>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>257</v>
       </c>
@@ -3959,7 +3959,7 @@
       <c r="C158" s="2"/>
       <c r="D158" s="2"/>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
         <v>258</v>
       </c>
@@ -3967,7 +3967,7 @@
       <c r="C159" s="2"/>
       <c r="D159" s="2"/>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
         <v>259</v>
       </c>
@@ -3975,7 +3975,7 @@
       <c r="C160" s="2"/>
       <c r="D160" s="2"/>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
         <v>260</v>
       </c>
@@ -3983,7 +3983,7 @@
       <c r="C161" s="2"/>
       <c r="D161" s="2"/>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>261</v>
       </c>
@@ -3991,7 +3991,7 @@
       <c r="C162" s="2"/>
       <c r="D162" s="2"/>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
         <v>262</v>
       </c>
@@ -3999,7 +3999,7 @@
       <c r="C163" s="2"/>
       <c r="D163" s="2"/>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
         <v>263</v>
       </c>
@@ -4007,7 +4007,7 @@
       <c r="C164" s="2"/>
       <c r="D164" s="2"/>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
         <v>279</v>
       </c>
@@ -4015,7 +4015,7 @@
       <c r="C165" s="2"/>
       <c r="D165" s="2"/>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
         <v>280</v>
       </c>
@@ -4023,7 +4023,7 @@
       <c r="C166" s="2"/>
       <c r="D166" s="2"/>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
         <v>281</v>
       </c>
@@ -4031,7 +4031,7 @@
       <c r="C167" s="2"/>
       <c r="D167" s="2"/>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
         <v>282</v>
       </c>
@@ -4039,7 +4039,7 @@
       <c r="C168" s="2"/>
       <c r="D168" s="2"/>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
         <v>283</v>
       </c>
@@ -4047,7 +4047,7 @@
       <c r="C169" s="2"/>
       <c r="D169" s="2"/>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
         <v>284</v>
       </c>
@@ -4055,7 +4055,7 @@
       <c r="C170" s="2"/>
       <c r="D170" s="2"/>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
         <v>285</v>
       </c>
@@ -4063,7 +4063,7 @@
       <c r="C171" s="2"/>
       <c r="D171" s="2"/>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
         <v>277</v>
       </c>
@@ -4071,7 +4071,7 @@
       <c r="C172" s="2"/>
       <c r="D172" s="2"/>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>271</v>
       </c>
@@ -4079,7 +4079,7 @@
       <c r="C173" s="2"/>
       <c r="D173" s="2"/>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
         <v>272</v>
       </c>
@@ -4087,7 +4087,7 @@
       <c r="C174" s="2"/>
       <c r="D174" s="2"/>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
         <v>273</v>
       </c>
@@ -4095,7 +4095,7 @@
       <c r="C175" s="2"/>
       <c r="D175" s="2"/>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
         <v>274</v>
       </c>
@@ -4103,7 +4103,7 @@
       <c r="C176" s="2"/>
       <c r="D176" s="2"/>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
         <v>275</v>
       </c>
@@ -4111,7 +4111,7 @@
       <c r="C177" s="2"/>
       <c r="D177" s="2"/>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
         <v>276</v>
       </c>
@@ -4119,7 +4119,7 @@
       <c r="C178" s="2"/>
       <c r="D178" s="2"/>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
         <v>140</v>
       </c>
@@ -4127,7 +4127,7 @@
       <c r="C179" s="2"/>
       <c r="D179" s="2"/>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>141</v>
       </c>
@@ -4135,7 +4135,7 @@
       <c r="C180" s="2"/>
       <c r="D180" s="2"/>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
         <v>142</v>
       </c>
@@ -4143,7 +4143,7 @@
       <c r="C181" s="2"/>
       <c r="D181" s="2"/>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
         <v>143</v>
       </c>
@@ -4151,7 +4151,7 @@
       <c r="C182" s="2"/>
       <c r="D182" s="2"/>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
         <v>144</v>
       </c>
@@ -4159,7 +4159,7 @@
       <c r="C183" s="2"/>
       <c r="D183" s="2"/>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
         <v>145</v>
       </c>
@@ -4167,7 +4167,7 @@
       <c r="C184" s="2"/>
       <c r="D184" s="2"/>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
         <v>146</v>
       </c>
@@ -4175,7 +4175,7 @@
       <c r="C185" s="2"/>
       <c r="D185" s="2"/>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
         <v>147</v>
       </c>
@@ -4183,7 +4183,7 @@
       <c r="C186" s="2"/>
       <c r="D186" s="2"/>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
         <v>148</v>
       </c>
@@ -4191,7 +4191,7 @@
       <c r="C187" s="2"/>
       <c r="D187" s="2"/>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
         <v>149</v>
       </c>
@@ -4199,7 +4199,7 @@
       <c r="C188" s="2"/>
       <c r="D188" s="2"/>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>150</v>
       </c>
@@ -4207,7 +4207,7 @@
       <c r="C189" s="2"/>
       <c r="D189" s="2"/>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
         <v>151</v>
       </c>
@@ -4215,7 +4215,7 @@
       <c r="C190" s="2"/>
       <c r="D190" s="2"/>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
         <v>152</v>
       </c>
@@ -4223,7 +4223,7 @@
       <c r="C191" s="2"/>
       <c r="D191" s="2"/>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
         <v>162</v>
       </c>
@@ -4231,7 +4231,7 @@
       <c r="C192" s="2"/>
       <c r="D192" s="2"/>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
         <v>163</v>
       </c>
@@ -4239,7 +4239,7 @@
       <c r="C193" s="2"/>
       <c r="D193" s="2"/>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
         <v>164</v>
       </c>
@@ -4247,7 +4247,7 @@
       <c r="C194" s="2"/>
       <c r="D194" s="2"/>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
         <v>165</v>
       </c>
@@ -4255,7 +4255,7 @@
       <c r="C195" s="2"/>
       <c r="D195" s="2"/>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
         <v>166</v>
       </c>
@@ -4263,7 +4263,7 @@
       <c r="C196" s="2"/>
       <c r="D196" s="2"/>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>167</v>
       </c>
@@ -4271,7 +4271,7 @@
       <c r="C197" s="2"/>
       <c r="D197" s="2"/>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
         <v>168</v>
       </c>
@@ -4279,7 +4279,7 @@
       <c r="C198" s="2"/>
       <c r="D198" s="2"/>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
         <v>198</v>
       </c>
@@ -4287,7 +4287,7 @@
       <c r="C199" s="2"/>
       <c r="D199" s="2"/>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
         <v>199</v>
       </c>
@@ -4295,7 +4295,7 @@
       <c r="C200" s="2"/>
       <c r="D200" s="2"/>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>223</v>
       </c>
@@ -4303,7 +4303,7 @@
       <c r="C201" s="2"/>
       <c r="D201" s="2"/>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
         <v>219</v>
       </c>
@@ -4311,7 +4311,7 @@
       <c r="C202" s="2"/>
       <c r="D202" s="2"/>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
         <v>220</v>
       </c>
@@ -4319,7 +4319,7 @@
       <c r="C203" s="2"/>
       <c r="D203" s="2"/>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
         <v>221</v>
       </c>
@@ -4327,7 +4327,7 @@
       <c r="C204" s="2"/>
       <c r="D204" s="2"/>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A205" s="2" t="s">
         <v>202</v>
       </c>
@@ -4335,7 +4335,7 @@
       <c r="C205" s="2"/>
       <c r="D205" s="2"/>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
         <v>203</v>
       </c>
@@ -4343,7 +4343,7 @@
       <c r="C206" s="2"/>
       <c r="D206" s="2"/>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
         <v>206</v>
       </c>
@@ -4351,7 +4351,7 @@
       <c r="C207" s="2"/>
       <c r="D207" s="2"/>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
         <v>207</v>
       </c>
@@ -4359,7 +4359,7 @@
       <c r="C208" s="2"/>
       <c r="D208" s="2"/>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
         <v>217</v>
       </c>
@@ -4367,7 +4367,7 @@
       <c r="C209" s="2"/>
       <c r="D209" s="2"/>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
         <v>286</v>
       </c>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="D210" s="2"/>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
         <v>287</v>
       </c>
@@ -4391,7 +4391,7 @@
       </c>
       <c r="D211" s="2"/>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
         <v>288</v>
       </c>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="D212" s="2"/>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
         <v>289</v>
       </c>
@@ -4415,7 +4415,7 @@
       </c>
       <c r="D213" s="2"/>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A214" s="2" t="s">
         <v>290</v>
       </c>
@@ -4427,7 +4427,7 @@
       </c>
       <c r="D214" s="2"/>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A215" s="2" t="s">
         <v>291</v>
       </c>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="D215" s="2"/>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
         <v>292</v>
       </c>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="D216" s="2"/>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A217" s="2" t="s">
         <v>293</v>
       </c>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="D217" s="2"/>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>294</v>
       </c>
@@ -4475,7 +4475,7 @@
       </c>
       <c r="D218" s="2"/>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
         <v>295</v>
       </c>
@@ -4487,7 +4487,7 @@
       </c>
       <c r="D219" s="2"/>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
         <v>212</v>
       </c>
@@ -4495,7 +4495,7 @@
       <c r="C220" s="2"/>
       <c r="D220" s="2"/>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
         <v>213</v>
       </c>
@@ -4503,7 +4503,7 @@
       <c r="C221" s="2"/>
       <c r="D221" s="2"/>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
         <v>301</v>
       </c>
@@ -4511,7 +4511,7 @@
       <c r="C222" s="2"/>
       <c r="D222" s="2"/>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>233</v>
       </c>
@@ -4519,7 +4519,7 @@
       <c r="C223" s="2"/>
       <c r="D223" s="2"/>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
         <v>264</v>
       </c>
@@ -4533,7 +4533,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A225" s="2" t="s">
         <v>265</v>
       </c>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="D225" s="2"/>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A226" s="2" t="s">
         <v>266</v>
       </c>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="D226" s="2"/>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A227" s="2" t="s">
         <v>267</v>
       </c>
@@ -4569,7 +4569,7 @@
       </c>
       <c r="D227" s="2"/>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
         <v>268</v>
       </c>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="D228" s="2"/>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
         <v>269</v>
       </c>
@@ -4593,7 +4593,7 @@
       </c>
       <c r="D229" s="2"/>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A230" s="2" t="s">
         <v>270</v>
       </c>

</xml_diff>